<commit_message>
V.1.1  Rapport completé jusqu'a la partie 3.2 (requêtes SQL)
</commit_message>
<xml_diff>
--- a/bases/BD_PAYS.xlsx
+++ b/bases/BD_PAYS.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kawyb\Desktop\L2 2K25\S4\Projet_bdd_sdd\bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kawyb\Desktop\projet_DataInvestigation\bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E41B23F-4506-4FA9-9D4F-A77773E1FD8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -3085,5 +3085,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>